<commit_message>
Resolved the ordering issue for team 1 in qualitative evaluation sheets
</commit_message>
<xml_diff>
--- a/evaluation/results/Qualitative Evaluations - System 1, System 2 and System 3/Evaluation-Sheet-mat.xlsx
+++ b/evaluation/results/Qualitative Evaluations - System 1, System 2 and System 3/Evaluation-Sheet-mat.xlsx
@@ -1,31 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27932"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DSouzaJ\Datasets\subject-indexing-dataset\evaluation\results\Qualitative Evaluations - System 1, System 2 and System 3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SadruddinS\Data\GermEval25\Qualitative Evaluations\Qualitative Evaluations-LA2I2F,DNB,ANNIF-updated\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{543C074A-A40A-4530-A03E-54D1475957FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19170" windowHeight="5910"/>
   </bookViews>
   <sheets>
     <sheet name="LLMs4Subjects Evaluation Sheet" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1871" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1871" uniqueCount="367">
   <si>
     <t>Record ID</t>
   </si>
@@ -882,6 +876,210 @@
     <t>Fläche | gnd:4129864-0</t>
   </si>
   <si>
+    <t>Homotopietheorie | gnd:4128142-1</t>
+  </si>
+  <si>
+    <t>Operatoralgebra | gnd:4129366-6</t>
+  </si>
+  <si>
+    <t>Linearer Operator | gnd:4167721-3</t>
+  </si>
+  <si>
+    <t>Derivation Algebra | gnd:4134656-7</t>
+  </si>
+  <si>
+    <t>Operatortheorie | gnd:4075665-8</t>
+  </si>
+  <si>
+    <t>AF-Algebra | gnd:4623947-9</t>
+  </si>
+  <si>
+    <t>Darstellungstheorie | gnd:4148816-7</t>
+  </si>
+  <si>
+    <t>Hilbert-Raum | gnd:4159850-7</t>
+  </si>
+  <si>
+    <t>Beschränkter Operator | gnd:4233452-4</t>
+  </si>
+  <si>
+    <t>Baer-Ring | gnd:4143902-8</t>
+  </si>
+  <si>
+    <t>Tensorprodukt | gnd:4059478-6</t>
+  </si>
+  <si>
+    <t>Selbstadjungierter Operator | gnd:4180810-1</t>
+  </si>
+  <si>
+    <t>Quantengruppe | gnd:4252437-4</t>
+  </si>
+  <si>
+    <t>Deformation Mathematik | gnd:4011284-6</t>
+  </si>
+  <si>
+    <t>Algebraische K-Theorie | gnd:4141839-6</t>
+  </si>
+  <si>
+    <t>Transformationsgruppe | gnd:4127386-2</t>
+  </si>
+  <si>
+    <t>Farrell-Jones-Vermutung | gnd:1172688117</t>
+  </si>
+  <si>
+    <t>Körper Algebra | gnd:4308063-7</t>
+  </si>
+  <si>
+    <t>Galois-Modul | gnd:4155898-4</t>
+  </si>
+  <si>
+    <t>Kommutative Algebra | gnd:4164821-3</t>
+  </si>
+  <si>
+    <t>Kategorientheorie | gnd:4120552-2</t>
+  </si>
+  <si>
+    <t>Fastring | gnd:4192482-4</t>
+  </si>
+  <si>
+    <t>Zensierte Stichprobe | gnd:4292948-9</t>
+  </si>
+  <si>
+    <t>Semiparametrisches Modell | gnd:4232479-8</t>
+  </si>
+  <si>
+    <t>Statistisches Funktional | gnd:4641370-4</t>
+  </si>
+  <si>
+    <t>Güte der Anpassung | gnd:4202143-1</t>
+  </si>
+  <si>
+    <t>Arbeitslosengeld II | gnd:4809112-1</t>
+  </si>
+  <si>
+    <t>Auswirkung | gnd:4112646-4</t>
+  </si>
+  <si>
+    <t>Mikrosimulation | gnd:4131395-1</t>
+  </si>
+  <si>
+    <t>Arbeitsloser | gnd:4002728-4</t>
+  </si>
+  <si>
+    <t>Arbeitsmarktpolitik | gnd:4002737-5</t>
+  </si>
+  <si>
+    <t>Hartz-Reform | gnd:4834482-5</t>
+  </si>
+  <si>
+    <t>Einkommen | gnd:4013887-2</t>
+  </si>
+  <si>
+    <t>Inzidenz Wirtschaft | gnd:4123447-9</t>
+  </si>
+  <si>
+    <t>Autoregressives Modell | gnd:4143717-2</t>
+  </si>
+  <si>
+    <t>Bewertung | gnd:4006340-9</t>
+  </si>
+  <si>
+    <t>State-Preference-Modell | gnd:4529201-2</t>
+  </si>
+  <si>
+    <t>Stochastischer Prozess | gnd:4057630-9</t>
+  </si>
+  <si>
+    <t>Derivat Wertpapier | gnd:4381572-8</t>
+  </si>
+  <si>
+    <t>Raum | gnd:4048561-4</t>
+  </si>
+  <si>
+    <t>Zeit | gnd:4067461-7</t>
+  </si>
+  <si>
+    <t>Lie-Gruppe | gnd:4035695-4</t>
+  </si>
+  <si>
+    <t>Symmetrie | gnd:4058724-1</t>
+  </si>
+  <si>
+    <t>Clifford-System | gnd:4148073-9</t>
+  </si>
+  <si>
+    <t>Anwendung | gnd:4196864-5</t>
+  </si>
+  <si>
+    <t>Maschinelles Sehen | gnd:4129594-8</t>
+  </si>
+  <si>
+    <t>Numerisches Verfahren | gnd:4128130-5</t>
+  </si>
+  <si>
+    <t>Euklidische Raumform | gnd:4804209-2</t>
+  </si>
+  <si>
+    <t>Raumgruppe | gnd:4177070-5</t>
+  </si>
+  <si>
+    <t>Clifford-Kleinsche Raumform | gnd:4228083-7</t>
+  </si>
+  <si>
+    <t>Multilineare Algebra | gnd:4416303-4</t>
+  </si>
+  <si>
+    <t>Mengenlehre | gnd:4074715-3</t>
+  </si>
+  <si>
+    <t>Homologie | gnd:4141951-0</t>
+  </si>
+  <si>
+    <t>Additive Semantik | gnd:4141386-6</t>
+  </si>
+  <si>
+    <t>Torsionstheorie | gnd:4451084-6</t>
+  </si>
+  <si>
+    <t>Quotientenring | gnd:4176745-7</t>
+  </si>
+  <si>
+    <t>Quotient | gnd:4312649-2</t>
+  </si>
+  <si>
+    <t>Kohomologietheorie | gnd:4164610-1</t>
+  </si>
+  <si>
+    <t>Homologische Algebra | gnd:4160598-6</t>
+  </si>
+  <si>
+    <t>Klassenkörper | gnd:4164021-4</t>
+  </si>
+  <si>
+    <t>Ordnung | gnd:4043744-9</t>
+  </si>
+  <si>
+    <t>Ordnungstheorie | gnd:4172736-8</t>
+  </si>
+  <si>
+    <t>LA2I2F - Team 1</t>
+  </si>
+  <si>
+    <t>Code</t>
+  </si>
+  <si>
+    <t>DNB-AI - Team 2</t>
+  </si>
+  <si>
+    <t>Annif - Team 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I </t>
+  </si>
+  <si>
+    <t>i</t>
+  </si>
+  <si>
     <t>Biochemische Methode | gnd:4319880-6</t>
   </si>
   <si>
@@ -922,213 +1120,12 @@
   </si>
   <si>
     <t>Bioinformatik | gnd:4611085-9</t>
-  </si>
-  <si>
-    <t>Homotopietheorie | gnd:4128142-1</t>
-  </si>
-  <si>
-    <t>Operatoralgebra | gnd:4129366-6</t>
-  </si>
-  <si>
-    <t>Linearer Operator | gnd:4167721-3</t>
-  </si>
-  <si>
-    <t>Derivation Algebra | gnd:4134656-7</t>
-  </si>
-  <si>
-    <t>Operatortheorie | gnd:4075665-8</t>
-  </si>
-  <si>
-    <t>AF-Algebra | gnd:4623947-9</t>
-  </si>
-  <si>
-    <t>Darstellungstheorie | gnd:4148816-7</t>
-  </si>
-  <si>
-    <t>Hilbert-Raum | gnd:4159850-7</t>
-  </si>
-  <si>
-    <t>Beschränkter Operator | gnd:4233452-4</t>
-  </si>
-  <si>
-    <t>Baer-Ring | gnd:4143902-8</t>
-  </si>
-  <si>
-    <t>Tensorprodukt | gnd:4059478-6</t>
-  </si>
-  <si>
-    <t>Selbstadjungierter Operator | gnd:4180810-1</t>
-  </si>
-  <si>
-    <t>Quantengruppe | gnd:4252437-4</t>
-  </si>
-  <si>
-    <t>Deformation Mathematik | gnd:4011284-6</t>
-  </si>
-  <si>
-    <t>Algebraische K-Theorie | gnd:4141839-6</t>
-  </si>
-  <si>
-    <t>Transformationsgruppe | gnd:4127386-2</t>
-  </si>
-  <si>
-    <t>Farrell-Jones-Vermutung | gnd:1172688117</t>
-  </si>
-  <si>
-    <t>Körper Algebra | gnd:4308063-7</t>
-  </si>
-  <si>
-    <t>Galois-Modul | gnd:4155898-4</t>
-  </si>
-  <si>
-    <t>Kommutative Algebra | gnd:4164821-3</t>
-  </si>
-  <si>
-    <t>Kategorientheorie | gnd:4120552-2</t>
-  </si>
-  <si>
-    <t>Fastring | gnd:4192482-4</t>
-  </si>
-  <si>
-    <t>Zensierte Stichprobe | gnd:4292948-9</t>
-  </si>
-  <si>
-    <t>Semiparametrisches Modell | gnd:4232479-8</t>
-  </si>
-  <si>
-    <t>Statistisches Funktional | gnd:4641370-4</t>
-  </si>
-  <si>
-    <t>Güte der Anpassung | gnd:4202143-1</t>
-  </si>
-  <si>
-    <t>Arbeitslosengeld II | gnd:4809112-1</t>
-  </si>
-  <si>
-    <t>Auswirkung | gnd:4112646-4</t>
-  </si>
-  <si>
-    <t>Mikrosimulation | gnd:4131395-1</t>
-  </si>
-  <si>
-    <t>Arbeitsloser | gnd:4002728-4</t>
-  </si>
-  <si>
-    <t>Arbeitsmarktpolitik | gnd:4002737-5</t>
-  </si>
-  <si>
-    <t>Hartz-Reform | gnd:4834482-5</t>
-  </si>
-  <si>
-    <t>Einkommen | gnd:4013887-2</t>
-  </si>
-  <si>
-    <t>Inzidenz Wirtschaft | gnd:4123447-9</t>
-  </si>
-  <si>
-    <t>Autoregressives Modell | gnd:4143717-2</t>
-  </si>
-  <si>
-    <t>Bewertung | gnd:4006340-9</t>
-  </si>
-  <si>
-    <t>State-Preference-Modell | gnd:4529201-2</t>
-  </si>
-  <si>
-    <t>Stochastischer Prozess | gnd:4057630-9</t>
-  </si>
-  <si>
-    <t>Derivat Wertpapier | gnd:4381572-8</t>
-  </si>
-  <si>
-    <t>Raum | gnd:4048561-4</t>
-  </si>
-  <si>
-    <t>Zeit | gnd:4067461-7</t>
-  </si>
-  <si>
-    <t>Lie-Gruppe | gnd:4035695-4</t>
-  </si>
-  <si>
-    <t>Symmetrie | gnd:4058724-1</t>
-  </si>
-  <si>
-    <t>Clifford-System | gnd:4148073-9</t>
-  </si>
-  <si>
-    <t>Anwendung | gnd:4196864-5</t>
-  </si>
-  <si>
-    <t>Maschinelles Sehen | gnd:4129594-8</t>
-  </si>
-  <si>
-    <t>Numerisches Verfahren | gnd:4128130-5</t>
-  </si>
-  <si>
-    <t>Euklidische Raumform | gnd:4804209-2</t>
-  </si>
-  <si>
-    <t>Raumgruppe | gnd:4177070-5</t>
-  </si>
-  <si>
-    <t>Clifford-Kleinsche Raumform | gnd:4228083-7</t>
-  </si>
-  <si>
-    <t>Multilineare Algebra | gnd:4416303-4</t>
-  </si>
-  <si>
-    <t>Mengenlehre | gnd:4074715-3</t>
-  </si>
-  <si>
-    <t>Homologie | gnd:4141951-0</t>
-  </si>
-  <si>
-    <t>Additive Semantik | gnd:4141386-6</t>
-  </si>
-  <si>
-    <t>Torsionstheorie | gnd:4451084-6</t>
-  </si>
-  <si>
-    <t>Quotientenring | gnd:4176745-7</t>
-  </si>
-  <si>
-    <t>Quotient | gnd:4312649-2</t>
-  </si>
-  <si>
-    <t>Kohomologietheorie | gnd:4164610-1</t>
-  </si>
-  <si>
-    <t>Homologische Algebra | gnd:4160598-6</t>
-  </si>
-  <si>
-    <t>Klassenkörper | gnd:4164021-4</t>
-  </si>
-  <si>
-    <t>Ordnung | gnd:4043744-9</t>
-  </si>
-  <si>
-    <t>Ordnungstheorie | gnd:4172736-8</t>
-  </si>
-  <si>
-    <t>Code</t>
-  </si>
-  <si>
-    <t xml:space="preserve">I </t>
-  </si>
-  <si>
-    <t>System 1</t>
-  </si>
-  <si>
-    <t>System 2</t>
-  </si>
-  <si>
-    <t>System 3</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1210,9 +1207,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1250,9 +1247,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1287,7 +1284,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1322,7 +1319,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1495,7 +1492,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:K201"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1529,22 +1526,22 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>363</v>
+        <v>347</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>361</v>
+        <v>348</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>364</v>
+        <v>349</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>361</v>
+        <v>348</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>365</v>
+        <v>350</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>361</v>
+        <v>348</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
@@ -3791,7 +3788,7 @@
         <v>282</v>
       </c>
       <c r="G76" t="s">
-        <v>362</v>
+        <v>351</v>
       </c>
       <c r="J76" t="s">
         <v>104</v>
@@ -3965,7 +3962,7 @@
         <v>285</v>
       </c>
       <c r="G82" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="H82" t="s">
         <v>111</v>
@@ -3997,10 +3994,10 @@
         <v>30</v>
       </c>
       <c r="F83" t="s">
-        <v>286</v>
+        <v>110</v>
       </c>
       <c r="G83" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="H83" t="s">
         <v>110</v>
@@ -4032,7 +4029,7 @@
         <v>30</v>
       </c>
       <c r="F84" t="s">
-        <v>211</v>
+        <v>111</v>
       </c>
       <c r="G84" t="s">
         <v>222</v>
@@ -4067,10 +4064,10 @@
         <v>30</v>
       </c>
       <c r="F85" t="s">
-        <v>202</v>
+        <v>286</v>
       </c>
       <c r="G85" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="H85" t="s">
         <v>113</v>
@@ -4102,10 +4099,10 @@
         <v>30</v>
       </c>
       <c r="F86" t="s">
-        <v>213</v>
+        <v>287</v>
       </c>
       <c r="G86" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="J86" t="s">
         <v>114</v>
@@ -4131,10 +4128,10 @@
         <v>30</v>
       </c>
       <c r="F87" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="G87" t="s">
-        <v>223</v>
+        <v>352</v>
       </c>
       <c r="J87" t="s">
         <v>115</v>
@@ -4160,7 +4157,7 @@
         <v>30</v>
       </c>
       <c r="F88" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="G88" t="s">
         <v>223</v>
@@ -4189,7 +4186,7 @@
         <v>30</v>
       </c>
       <c r="F89" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="G89" t="s">
         <v>223</v>
@@ -4218,7 +4215,7 @@
         <v>30</v>
       </c>
       <c r="F90" t="s">
-        <v>290</v>
+        <v>118</v>
       </c>
       <c r="G90" t="s">
         <v>223</v>
@@ -4247,10 +4244,10 @@
         <v>30</v>
       </c>
       <c r="F91" t="s">
-        <v>218</v>
+        <v>291</v>
       </c>
       <c r="G91" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="J91" t="s">
         <v>119</v>
@@ -4276,7 +4273,7 @@
         <v>30</v>
       </c>
       <c r="F92" t="s">
-        <v>291</v>
+        <v>134</v>
       </c>
       <c r="G92" t="s">
         <v>223</v>
@@ -4305,10 +4302,10 @@
         <v>30</v>
       </c>
       <c r="F93" t="s">
-        <v>203</v>
+        <v>292</v>
       </c>
       <c r="G93" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="J93" t="s">
         <v>121</v>
@@ -4334,10 +4331,10 @@
         <v>30</v>
       </c>
       <c r="F94" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="G94" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="J94" t="s">
         <v>122</v>
@@ -4363,7 +4360,7 @@
         <v>30</v>
       </c>
       <c r="F95" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="G95" t="s">
         <v>223</v>
@@ -4392,10 +4389,10 @@
         <v>30</v>
       </c>
       <c r="F96" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="G96" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="J96" t="s">
         <v>124</v>
@@ -4421,10 +4418,10 @@
         <v>30</v>
       </c>
       <c r="F97" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="G97" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="J97" t="s">
         <v>125</v>
@@ -4450,7 +4447,7 @@
         <v>30</v>
       </c>
       <c r="F98" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="G98" t="s">
         <v>223</v>
@@ -4479,10 +4476,10 @@
         <v>30</v>
       </c>
       <c r="F99" t="s">
-        <v>297</v>
+        <v>114</v>
       </c>
       <c r="G99" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="J99" t="s">
         <v>127</v>
@@ -4508,10 +4505,10 @@
         <v>30</v>
       </c>
       <c r="F100" t="s">
-        <v>298</v>
+        <v>273</v>
       </c>
       <c r="G100" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="J100" t="s">
         <v>128</v>
@@ -4537,7 +4534,7 @@
         <v>30</v>
       </c>
       <c r="F101" t="s">
-        <v>196</v>
+        <v>298</v>
       </c>
       <c r="G101" t="s">
         <v>222</v>
@@ -4566,7 +4563,7 @@
         <v>30</v>
       </c>
       <c r="F102" t="s">
-        <v>299</v>
+        <v>132</v>
       </c>
       <c r="G102" t="s">
         <v>221</v>
@@ -4601,10 +4598,10 @@
         <v>30</v>
       </c>
       <c r="F103" t="s">
-        <v>110</v>
+        <v>148</v>
       </c>
       <c r="G103" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="J103" t="s">
         <v>131</v>
@@ -4630,10 +4627,10 @@
         <v>30</v>
       </c>
       <c r="F104" t="s">
-        <v>111</v>
+        <v>336</v>
       </c>
       <c r="G104" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="J104" t="s">
         <v>132</v>
@@ -4659,10 +4656,10 @@
         <v>30</v>
       </c>
       <c r="F105" t="s">
-        <v>300</v>
+        <v>337</v>
       </c>
       <c r="G105" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="J105" t="s">
         <v>133</v>
@@ -4688,10 +4685,10 @@
         <v>30</v>
       </c>
       <c r="F106" t="s">
-        <v>301</v>
+        <v>134</v>
       </c>
       <c r="G106" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="J106" t="s">
         <v>134</v>
@@ -4717,10 +4714,10 @@
         <v>30</v>
       </c>
       <c r="F107" t="s">
-        <v>302</v>
+        <v>338</v>
       </c>
       <c r="G107" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="J107" t="s">
         <v>135</v>
@@ -4746,10 +4743,10 @@
         <v>30</v>
       </c>
       <c r="F108" t="s">
-        <v>303</v>
+        <v>339</v>
       </c>
       <c r="G108" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="J108" t="s">
         <v>136</v>
@@ -4775,10 +4772,10 @@
         <v>30</v>
       </c>
       <c r="F109" t="s">
-        <v>304</v>
+        <v>340</v>
       </c>
       <c r="G109" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="J109" t="s">
         <v>137</v>
@@ -4804,10 +4801,10 @@
         <v>30</v>
       </c>
       <c r="F110" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="G110" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="J110" t="s">
         <v>138</v>
@@ -4833,10 +4830,10 @@
         <v>30</v>
       </c>
       <c r="F111" t="s">
-        <v>305</v>
+        <v>130</v>
       </c>
       <c r="G111" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="J111" t="s">
         <v>139</v>
@@ -4862,7 +4859,7 @@
         <v>30</v>
       </c>
       <c r="F112" t="s">
-        <v>134</v>
+        <v>155</v>
       </c>
       <c r="G112" t="s">
         <v>223</v>
@@ -4891,10 +4888,10 @@
         <v>30</v>
       </c>
       <c r="F113" t="s">
-        <v>306</v>
+        <v>341</v>
       </c>
       <c r="G113" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="J113" t="s">
         <v>141</v>
@@ -4920,7 +4917,7 @@
         <v>30</v>
       </c>
       <c r="F114" t="s">
-        <v>307</v>
+        <v>342</v>
       </c>
       <c r="G114" t="s">
         <v>221</v>
@@ -4949,10 +4946,10 @@
         <v>30</v>
       </c>
       <c r="F115" t="s">
-        <v>308</v>
+        <v>142</v>
       </c>
       <c r="G115" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="J115" t="s">
         <v>143</v>
@@ -4978,7 +4975,7 @@
         <v>30</v>
       </c>
       <c r="F116" t="s">
-        <v>309</v>
+        <v>343</v>
       </c>
       <c r="G116" t="s">
         <v>221</v>
@@ -5007,7 +5004,7 @@
         <v>30</v>
       </c>
       <c r="F117" t="s">
-        <v>310</v>
+        <v>111</v>
       </c>
       <c r="G117" t="s">
         <v>223</v>
@@ -5036,7 +5033,7 @@
         <v>30</v>
       </c>
       <c r="F118" t="s">
-        <v>311</v>
+        <v>344</v>
       </c>
       <c r="G118" t="s">
         <v>223</v>
@@ -5065,7 +5062,7 @@
         <v>30</v>
       </c>
       <c r="F119" t="s">
-        <v>114</v>
+        <v>345</v>
       </c>
       <c r="G119" t="s">
         <v>221</v>
@@ -5094,10 +5091,10 @@
         <v>30</v>
       </c>
       <c r="F120" t="s">
-        <v>273</v>
+        <v>33</v>
       </c>
       <c r="G120" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="J120" t="s">
         <v>148</v>
@@ -5123,10 +5120,10 @@
         <v>30</v>
       </c>
       <c r="F121" t="s">
-        <v>312</v>
+        <v>346</v>
       </c>
       <c r="G121" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="J121" t="s">
         <v>149</v>
@@ -5152,7 +5149,7 @@
         <v>30</v>
       </c>
       <c r="F122" t="s">
-        <v>305</v>
+        <v>291</v>
       </c>
       <c r="G122" t="s">
         <v>223</v>
@@ -5222,7 +5219,7 @@
         <v>30</v>
       </c>
       <c r="F124" t="s">
-        <v>313</v>
+        <v>299</v>
       </c>
       <c r="G124" t="s">
         <v>223</v>
@@ -5257,7 +5254,7 @@
         <v>30</v>
       </c>
       <c r="F125" t="s">
-        <v>314</v>
+        <v>300</v>
       </c>
       <c r="G125" t="s">
         <v>223</v>
@@ -5286,7 +5283,7 @@
         <v>30</v>
       </c>
       <c r="F126" t="s">
-        <v>315</v>
+        <v>301</v>
       </c>
       <c r="G126" t="s">
         <v>223</v>
@@ -5489,7 +5486,7 @@
         <v>30</v>
       </c>
       <c r="F133" t="s">
-        <v>316</v>
+        <v>302</v>
       </c>
       <c r="G133" t="s">
         <v>223</v>
@@ -5547,7 +5544,7 @@
         <v>30</v>
       </c>
       <c r="F135" t="s">
-        <v>317</v>
+        <v>303</v>
       </c>
       <c r="G135" t="s">
         <v>223</v>
@@ -5663,7 +5660,7 @@
         <v>30</v>
       </c>
       <c r="F139" t="s">
-        <v>318</v>
+        <v>304</v>
       </c>
       <c r="G139" t="s">
         <v>223</v>
@@ -5692,7 +5689,7 @@
         <v>30</v>
       </c>
       <c r="F140" t="s">
-        <v>319</v>
+        <v>305</v>
       </c>
       <c r="G140" t="s">
         <v>223</v>
@@ -5721,7 +5718,7 @@
         <v>30</v>
       </c>
       <c r="F141" t="s">
-        <v>320</v>
+        <v>306</v>
       </c>
       <c r="G141" t="s">
         <v>223</v>
@@ -5785,7 +5782,7 @@
         <v>30</v>
       </c>
       <c r="F143" t="s">
-        <v>321</v>
+        <v>307</v>
       </c>
       <c r="G143" t="s">
         <v>223</v>
@@ -5820,7 +5817,7 @@
         <v>30</v>
       </c>
       <c r="F144" t="s">
-        <v>322</v>
+        <v>308</v>
       </c>
       <c r="G144" t="s">
         <v>223</v>
@@ -5855,7 +5852,7 @@
         <v>30</v>
       </c>
       <c r="F145" t="s">
-        <v>323</v>
+        <v>309</v>
       </c>
       <c r="G145" t="s">
         <v>223</v>
@@ -5884,7 +5881,7 @@
         <v>30</v>
       </c>
       <c r="F146" t="s">
-        <v>324</v>
+        <v>310</v>
       </c>
       <c r="G146" t="s">
         <v>223</v>
@@ -5913,7 +5910,7 @@
         <v>30</v>
       </c>
       <c r="F147" t="s">
-        <v>325</v>
+        <v>311</v>
       </c>
       <c r="G147" t="s">
         <v>223</v>
@@ -5942,7 +5939,7 @@
         <v>30</v>
       </c>
       <c r="F148" t="s">
-        <v>326</v>
+        <v>312</v>
       </c>
       <c r="G148" t="s">
         <v>223</v>
@@ -5971,7 +5968,7 @@
         <v>30</v>
       </c>
       <c r="F149" t="s">
-        <v>327</v>
+        <v>313</v>
       </c>
       <c r="G149" t="s">
         <v>223</v>
@@ -6000,7 +5997,7 @@
         <v>30</v>
       </c>
       <c r="F150" t="s">
-        <v>328</v>
+        <v>314</v>
       </c>
       <c r="G150" t="s">
         <v>223</v>
@@ -6029,7 +6026,7 @@
         <v>30</v>
       </c>
       <c r="F151" t="s">
-        <v>329</v>
+        <v>315</v>
       </c>
       <c r="G151" t="s">
         <v>223</v>
@@ -6058,7 +6055,7 @@
         <v>30</v>
       </c>
       <c r="F152" t="s">
-        <v>330</v>
+        <v>316</v>
       </c>
       <c r="G152" t="s">
         <v>223</v>
@@ -6087,7 +6084,7 @@
         <v>30</v>
       </c>
       <c r="F153" t="s">
-        <v>331</v>
+        <v>317</v>
       </c>
       <c r="G153" t="s">
         <v>223</v>
@@ -6116,7 +6113,7 @@
         <v>30</v>
       </c>
       <c r="F154" t="s">
-        <v>332</v>
+        <v>318</v>
       </c>
       <c r="G154" t="s">
         <v>223</v>
@@ -6145,7 +6142,7 @@
         <v>30</v>
       </c>
       <c r="F155" t="s">
-        <v>333</v>
+        <v>319</v>
       </c>
       <c r="G155" t="s">
         <v>223</v>
@@ -6203,7 +6200,7 @@
         <v>30</v>
       </c>
       <c r="F157" t="s">
-        <v>334</v>
+        <v>320</v>
       </c>
       <c r="G157" t="s">
         <v>223</v>
@@ -6232,7 +6229,7 @@
         <v>30</v>
       </c>
       <c r="F158" t="s">
-        <v>335</v>
+        <v>321</v>
       </c>
       <c r="G158" t="s">
         <v>223</v>
@@ -6261,7 +6258,7 @@
         <v>30</v>
       </c>
       <c r="F159" t="s">
-        <v>336</v>
+        <v>322</v>
       </c>
       <c r="G159" t="s">
         <v>223</v>
@@ -6290,7 +6287,7 @@
         <v>30</v>
       </c>
       <c r="F160" t="s">
-        <v>337</v>
+        <v>323</v>
       </c>
       <c r="G160" t="s">
         <v>223</v>
@@ -6453,7 +6450,7 @@
         <v>30</v>
       </c>
       <c r="F165" t="s">
-        <v>338</v>
+        <v>324</v>
       </c>
       <c r="G165" t="s">
         <v>223</v>
@@ -6482,7 +6479,7 @@
         <v>30</v>
       </c>
       <c r="F166" t="s">
-        <v>339</v>
+        <v>325</v>
       </c>
       <c r="G166" t="s">
         <v>223</v>
@@ -6511,7 +6508,7 @@
         <v>30</v>
       </c>
       <c r="F167" t="s">
-        <v>340</v>
+        <v>326</v>
       </c>
       <c r="G167" t="s">
         <v>223</v>
@@ -6569,7 +6566,7 @@
         <v>30</v>
       </c>
       <c r="F169" t="s">
-        <v>341</v>
+        <v>327</v>
       </c>
       <c r="G169" t="s">
         <v>223</v>
@@ -6627,7 +6624,7 @@
         <v>30</v>
       </c>
       <c r="F171" t="s">
-        <v>342</v>
+        <v>328</v>
       </c>
       <c r="G171" t="s">
         <v>223</v>
@@ -6656,7 +6653,7 @@
         <v>30</v>
       </c>
       <c r="F172" t="s">
-        <v>343</v>
+        <v>329</v>
       </c>
       <c r="G172" t="s">
         <v>223</v>
@@ -6714,7 +6711,7 @@
         <v>30</v>
       </c>
       <c r="F174" t="s">
-        <v>344</v>
+        <v>330</v>
       </c>
       <c r="G174" t="s">
         <v>223</v>
@@ -6743,7 +6740,7 @@
         <v>30</v>
       </c>
       <c r="F175" t="s">
-        <v>345</v>
+        <v>331</v>
       </c>
       <c r="G175" t="s">
         <v>223</v>
@@ -6772,7 +6769,7 @@
         <v>30</v>
       </c>
       <c r="F176" t="s">
-        <v>346</v>
+        <v>332</v>
       </c>
       <c r="G176" t="s">
         <v>223</v>
@@ -6801,7 +6798,7 @@
         <v>30</v>
       </c>
       <c r="F177" t="s">
-        <v>305</v>
+        <v>291</v>
       </c>
       <c r="G177" t="s">
         <v>223</v>
@@ -6830,7 +6827,7 @@
         <v>30</v>
       </c>
       <c r="F178" t="s">
-        <v>347</v>
+        <v>333</v>
       </c>
       <c r="G178" t="s">
         <v>223</v>
@@ -6859,7 +6856,7 @@
         <v>30</v>
       </c>
       <c r="F179" t="s">
-        <v>348</v>
+        <v>334</v>
       </c>
       <c r="G179" t="s">
         <v>223</v>
@@ -6888,7 +6885,7 @@
         <v>30</v>
       </c>
       <c r="F180" t="s">
-        <v>349</v>
+        <v>335</v>
       </c>
       <c r="G180" t="s">
         <v>223</v>
@@ -6946,10 +6943,10 @@
         <v>32</v>
       </c>
       <c r="F182" t="s">
-        <v>132</v>
+        <v>353</v>
       </c>
       <c r="G182" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="H182" t="s">
         <v>202</v>
@@ -6981,7 +6978,7 @@
         <v>32</v>
       </c>
       <c r="F183" t="s">
-        <v>148</v>
+        <v>354</v>
       </c>
       <c r="G183" t="s">
         <v>223</v>
@@ -7016,10 +7013,10 @@
         <v>32</v>
       </c>
       <c r="F184" t="s">
-        <v>350</v>
+        <v>211</v>
       </c>
       <c r="G184" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="H184" t="s">
         <v>213</v>
@@ -7051,10 +7048,10 @@
         <v>32</v>
       </c>
       <c r="F185" t="s">
-        <v>351</v>
+        <v>202</v>
       </c>
       <c r="G185" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="J185" t="s">
         <v>204</v>
@@ -7080,7 +7077,7 @@
         <v>32</v>
       </c>
       <c r="F186" t="s">
-        <v>134</v>
+        <v>213</v>
       </c>
       <c r="G186" t="s">
         <v>222</v>
@@ -7109,7 +7106,7 @@
         <v>32</v>
       </c>
       <c r="F187" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="G187" t="s">
         <v>223</v>
@@ -7138,10 +7135,10 @@
         <v>32</v>
       </c>
       <c r="F188" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="G188" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="J188" t="s">
         <v>207</v>
@@ -7167,10 +7164,10 @@
         <v>32</v>
       </c>
       <c r="F189" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="G189" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="J189" t="s">
         <v>208</v>
@@ -7196,10 +7193,10 @@
         <v>32</v>
       </c>
       <c r="F190" t="s">
-        <v>126</v>
+        <v>358</v>
       </c>
       <c r="G190" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="J190" t="s">
         <v>209</v>
@@ -7225,7 +7222,7 @@
         <v>32</v>
       </c>
       <c r="F191" t="s">
-        <v>130</v>
+        <v>218</v>
       </c>
       <c r="G191" t="s">
         <v>222</v>
@@ -7254,7 +7251,7 @@
         <v>32</v>
       </c>
       <c r="F192" t="s">
-        <v>155</v>
+        <v>359</v>
       </c>
       <c r="G192" t="s">
         <v>223</v>
@@ -7283,10 +7280,10 @@
         <v>32</v>
       </c>
       <c r="F193" t="s">
-        <v>355</v>
+        <v>203</v>
       </c>
       <c r="G193" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="J193" t="s">
         <v>212</v>
@@ -7312,10 +7309,10 @@
         <v>32</v>
       </c>
       <c r="F194" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="G194" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="J194" t="s">
         <v>213</v>
@@ -7341,10 +7338,10 @@
         <v>32</v>
       </c>
       <c r="F195" t="s">
-        <v>142</v>
+        <v>361</v>
       </c>
       <c r="G195" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="J195" t="s">
         <v>214</v>
@@ -7370,10 +7367,10 @@
         <v>32</v>
       </c>
       <c r="F196" t="s">
-        <v>357</v>
+        <v>362</v>
       </c>
       <c r="G196" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="J196" t="s">
         <v>215</v>
@@ -7399,10 +7396,10 @@
         <v>32</v>
       </c>
       <c r="F197" t="s">
-        <v>111</v>
+        <v>363</v>
       </c>
       <c r="G197" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="J197" t="s">
         <v>216</v>
@@ -7428,7 +7425,7 @@
         <v>32</v>
       </c>
       <c r="F198" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
       <c r="G198" t="s">
         <v>223</v>
@@ -7457,10 +7454,10 @@
         <v>32</v>
       </c>
       <c r="F199" t="s">
-        <v>359</v>
+        <v>365</v>
       </c>
       <c r="G199" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="J199" t="s">
         <v>218</v>
@@ -7486,10 +7483,10 @@
         <v>32</v>
       </c>
       <c r="F200" t="s">
-        <v>33</v>
+        <v>366</v>
       </c>
       <c r="G200" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="J200" t="s">
         <v>219</v>
@@ -7515,10 +7512,10 @@
         <v>32</v>
       </c>
       <c r="F201" t="s">
-        <v>360</v>
+        <v>196</v>
       </c>
       <c r="G201" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="J201" t="s">
         <v>220</v>

</xml_diff>